<commit_message>
chore: full dashboard refresh (Jul 2026) — data, analytics, intelligence report, QA
</commit_message>
<xml_diff>
--- a/inputs/Output-Indicator-Lookup.xlsx
+++ b/inputs/Output-Indicator-Lookup.xlsx
@@ -13,7 +13,7 @@
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20960" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Indicator Lookup" sheetId="9" r:id="rId6"/>
+    <sheet name="Indicator Lookup" sheetId="13" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="true"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="952">
   <si>
     <t>Latest Period</t>
   </si>
@@ -1443,6 +1443,1428 @@
   </si>
   <si>
     <t>Disability Support Pension</t>
+  </si>
+  <si>
+    <t>Tourism</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>STRA</t>
+  </si>
+  <si>
+    <t>Airbnb Occupancy Rate</t>
+  </si>
+  <si>
+    <t>Latest Period</t>
+  </si>
+  <si>
+    <t>Content Area</t>
+  </si>
+  <si>
+    <t>Data Frequency</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>Indicator</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Property Market</t>
+  </si>
+  <si>
+    <t>Unit Price (Current)</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Retail Spend</t>
+  </si>
+  <si>
+    <t>Total Spend</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>% Bachelor Degree</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Count of Business</t>
+  </si>
+  <si>
+    <t>Tourism Businesses</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Median Household Income</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Property Market</t>
+  </si>
+  <si>
+    <t>Unit Rent (P/W)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>Population density 2024 (persons/km2)</t>
+  </si>
+  <si>
+    <t>Crime</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>BOCSAR</t>
+  </si>
+  <si>
+    <t>Assault Rate (per 1,000)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>Natural increase in ERP</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Median Age</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Property Market</t>
+  </si>
+  <si>
+    <t>Listing Visits per Property</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Family Tax Benefit A</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Count of Business</t>
+  </si>
+  <si>
+    <t>Total Businesses</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Commonwealth Rent Assistance</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Carer Allowance</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>SALM</t>
+  </si>
+  <si>
+    <t>Unemployment</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Total Indigenous</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>ERP Change 2023-24</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>ABS Population</t>
+  </si>
+  <si>
+    <t>% Under 20</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Total Population</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>% ERP Change 2023-24</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Age Pension</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>% Indigenous</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>% Language Other Than English</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>SALM</t>
+  </si>
+  <si>
+    <t>Unemployment Rate (%)</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>JobSeeker</t>
+  </si>
+  <si>
+    <t>Youth Allowance (other)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>ABS Population</t>
+  </si>
+  <si>
+    <t>% Over 69</t>
+  </si>
+  <si>
+    <t>Tourism</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>STRA</t>
+  </si>
+  <si>
+    <t>Airbnb ADR</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>Net internal migration</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>% Born Overseas</t>
+  </si>
+  <si>
+    <t>Tourism</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>STRA</t>
+  </si>
+  <si>
+    <t>Airbnb Active Listings</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Pension Concession Card</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>% Completed Year 12</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Parenting Payment Single</t>
+  </si>
+  <si>
+    <t>Crime</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>BOCSAR</t>
+  </si>
+  <si>
+    <t>Malicious Damage to Property Rate (per 1,000)</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Disability Support Pension</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>ERP at 30 June 2023</t>
+  </si>
+  <si>
+    <t>Crime</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>BOCSAR</t>
+  </si>
+  <si>
+    <t>Drug Offences Rate (per 1,000)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Index of Relative Socio-economic Advantage and Disadvantage</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Property Market</t>
+  </si>
+  <si>
+    <t>House Price (Current)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Index of Relative Socio-economic Disadvantage </t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Index of Economic Resources</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>Net overseas migration</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Count of Business</t>
+  </si>
+  <si>
+    <t>Manufacturing Businesses</t>
+  </si>
+  <si>
+    <t>Housing</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Building Approvals</t>
+  </si>
+  <si>
+    <t>Value of building job(s)</t>
+  </si>
+  <si>
+    <t>Tourism</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>STRA</t>
+  </si>
+  <si>
+    <t>Airbnb  Gross Revenue</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Index of Education and Occupation</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>SALM</t>
+  </si>
+  <si>
+    <t>Labour Force</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Health Care Card</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>JobSeeker</t>
+  </si>
+  <si>
+    <t>JobSeeker Payment</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Homelessness (AIHW)</t>
+  </si>
+  <si>
+    <t>Homelessness</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Count of Business</t>
+  </si>
+  <si>
+    <t>Healthcare Businesses</t>
+  </si>
+  <si>
+    <t>Crime</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>BOCSAR</t>
+  </si>
+  <si>
+    <t>Theft Rate (per 1,000)</t>
+  </si>
+  <si>
+    <t>Housing</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Building Approvals</t>
+  </si>
+  <si>
+    <t>Number of dwellings approved</t>
+  </si>
+  <si>
+    <t>Crime</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>BOCSAR</t>
+  </si>
+  <si>
+    <t>Intimidation, Stalking &amp; Harassment Rate (per 1,000)</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Property Market</t>
+  </si>
+  <si>
+    <t>House Rent (P/W)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>ERP at 30 June 2024</t>
+  </si>
+  <si>
+    <t>Tourism</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>STRA</t>
+  </si>
+  <si>
+    <t>Airbnb Occupancy Rate</t>
+  </si>
+  <si>
+    <t>Latest Period</t>
+  </si>
+  <si>
+    <t>Content Area</t>
+  </si>
+  <si>
+    <t>Data Frequency</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>Indicator</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Property Market</t>
+  </si>
+  <si>
+    <t>Unit Price (Current)</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Retail Spend</t>
+  </si>
+  <si>
+    <t>Total Spend</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>% Bachelor Degree</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Count of Business</t>
+  </si>
+  <si>
+    <t>Tourism Businesses</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Median Household Income</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Property Market</t>
+  </si>
+  <si>
+    <t>Unit Rent (P/W)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>Population density 2024 (persons/km2)</t>
+  </si>
+  <si>
+    <t>Crime</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>BOCSAR</t>
+  </si>
+  <si>
+    <t>Assault Rate (per 1,000)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>Natural increase in ERP</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Median Age</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Property Market</t>
+  </si>
+  <si>
+    <t>Listing Visits per Property</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Family Tax Benefit A</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Count of Business</t>
+  </si>
+  <si>
+    <t>Total Businesses</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Commonwealth Rent Assistance</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Carer Allowance</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>SALM</t>
+  </si>
+  <si>
+    <t>Unemployment</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Total Indigenous</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>ERP Change 2023-24</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>ABS Population</t>
+  </si>
+  <si>
+    <t>% Under 20</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Total Population</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>% ERP Change 2023-24</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Age Pension</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>% Indigenous</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>% Language Other Than English</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>SALM</t>
+  </si>
+  <si>
+    <t>Unemployment Rate (%)</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>JobSeeker</t>
+  </si>
+  <si>
+    <t>Youth Allowance (other)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>ABS Population</t>
+  </si>
+  <si>
+    <t>% Over 69</t>
+  </si>
+  <si>
+    <t>Tourism</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>STRA</t>
+  </si>
+  <si>
+    <t>Airbnb ADR</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>Net internal migration</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>% Born Overseas</t>
+  </si>
+  <si>
+    <t>Tourism</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>STRA</t>
+  </si>
+  <si>
+    <t>Airbnb Active Listings</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Pension Concession Card</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>% Completed Year 12</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Parenting Payment Single</t>
+  </si>
+  <si>
+    <t>Crime</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>BOCSAR</t>
+  </si>
+  <si>
+    <t>Malicious Damage to Property Rate (per 1,000)</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Disability Support Pension</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>ERP at 30 June 2023</t>
+  </si>
+  <si>
+    <t>Crime</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>BOCSAR</t>
+  </si>
+  <si>
+    <t>Drug Offences Rate (per 1,000)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Index of Relative Socio-economic Advantage and Disadvantage</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Property Market</t>
+  </si>
+  <si>
+    <t>House Price (Current)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Index of Relative Socio-economic Disadvantage </t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Index of Economic Resources</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>Net overseas migration</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Count of Business</t>
+  </si>
+  <si>
+    <t>Manufacturing Businesses</t>
+  </si>
+  <si>
+    <t>Housing</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Building Approvals</t>
+  </si>
+  <si>
+    <t>Value of building job(s)</t>
+  </si>
+  <si>
+    <t>Tourism</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>STRA</t>
+  </si>
+  <si>
+    <t>Airbnb  Gross Revenue</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>4 Yearly</t>
+  </si>
+  <si>
+    <t>ABS Census</t>
+  </si>
+  <si>
+    <t>Index of Education and Occupation</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>SALM</t>
+  </si>
+  <si>
+    <t>Labour Force</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>DSS</t>
+  </si>
+  <si>
+    <t>Health Care Card</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>JobSeeker</t>
+  </si>
+  <si>
+    <t>JobSeeker Payment</t>
+  </si>
+  <si>
+    <t>Socio-Economic</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Homelessness (AIHW)</t>
+  </si>
+  <si>
+    <t>Homelessness</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Count of Business</t>
+  </si>
+  <si>
+    <t>Healthcare Businesses</t>
+  </si>
+  <si>
+    <t>Crime</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>BOCSAR</t>
+  </si>
+  <si>
+    <t>Theft Rate (per 1,000)</t>
+  </si>
+  <si>
+    <t>Housing</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Building Approvals</t>
+  </si>
+  <si>
+    <t>Number of dwellings approved</t>
+  </si>
+  <si>
+    <t>Crime</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>BOCSAR</t>
+  </si>
+  <si>
+    <t>Intimidation, Stalking &amp; Harassment Rate (per 1,000)</t>
+  </si>
+  <si>
+    <t>Economy</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Property Market</t>
+  </si>
+  <si>
+    <t>House Rent (P/W)</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Regional Population</t>
+  </si>
+  <si>
+    <t>ERP at 30 June 2024</t>
   </si>
   <si>
     <t>Tourism</t>
@@ -1475,7 +2897,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1492,15 +2914,23 @@
     </border>
     <border/>
     <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true" applyBorder="true"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="46" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1833,1012 +3263,1012 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>241</v>
+        <v>715</v>
       </c>
       <c r="B1" t="s">
-        <v>242</v>
+        <v>716</v>
       </c>
       <c r="C1" t="s">
-        <v>243</v>
+        <v>717</v>
       </c>
       <c r="D1" t="s">
-        <v>244</v>
+        <v>718</v>
       </c>
       <c r="E1" t="s">
-        <v>245</v>
+        <v>719</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="6">
+        <v>46204</v>
+      </c>
+      <c r="B2" t="s">
+        <v>720</v>
+      </c>
+      <c r="C2" t="s">
+        <v>721</v>
+      </c>
+      <c r="D2" t="s">
+        <v>722</v>
+      </c>
+      <c r="E2" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6">
         <v>46174</v>
       </c>
-      <c r="B2" t="s">
-        <v>246</v>
-      </c>
-      <c r="C2" t="s">
-        <v>247</v>
-      </c>
-      <c r="D2" t="s">
-        <v>248</v>
-      </c>
-      <c r="E2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
+      <c r="B3" t="s">
+        <v>724</v>
+      </c>
+      <c r="C3" t="s">
+        <v>725</v>
+      </c>
+      <c r="D3" t="s">
+        <v>726</v>
+      </c>
+      <c r="E3" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6">
+        <v>44377</v>
+      </c>
+      <c r="B4" t="s">
+        <v>728</v>
+      </c>
+      <c r="C4" t="s">
+        <v>729</v>
+      </c>
+      <c r="D4" t="s">
+        <v>730</v>
+      </c>
+      <c r="E4" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6">
+        <v>45658</v>
+      </c>
+      <c r="B5" t="s">
+        <v>732</v>
+      </c>
+      <c r="C5" t="s">
+        <v>733</v>
+      </c>
+      <c r="D5" t="s">
+        <v>734</v>
+      </c>
+      <c r="E5" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6">
+        <v>44377</v>
+      </c>
+      <c r="B6" t="s">
+        <v>736</v>
+      </c>
+      <c r="C6" t="s">
+        <v>737</v>
+      </c>
+      <c r="D6" t="s">
+        <v>738</v>
+      </c>
+      <c r="E6" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6">
+        <v>46204</v>
+      </c>
+      <c r="B7" t="s">
+        <v>740</v>
+      </c>
+      <c r="C7" t="s">
+        <v>741</v>
+      </c>
+      <c r="D7" t="s">
+        <v>742</v>
+      </c>
+      <c r="E7" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6">
+        <v>45473</v>
+      </c>
+      <c r="B8" t="s">
+        <v>744</v>
+      </c>
+      <c r="C8" t="s">
+        <v>745</v>
+      </c>
+      <c r="D8" t="s">
+        <v>746</v>
+      </c>
+      <c r="E8" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6">
+        <v>46022</v>
+      </c>
+      <c r="B9" t="s">
+        <v>748</v>
+      </c>
+      <c r="C9" t="s">
+        <v>749</v>
+      </c>
+      <c r="D9" t="s">
+        <v>750</v>
+      </c>
+      <c r="E9" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6">
+        <v>45473</v>
+      </c>
+      <c r="B10" t="s">
+        <v>752</v>
+      </c>
+      <c r="C10" t="s">
+        <v>753</v>
+      </c>
+      <c r="D10" t="s">
+        <v>754</v>
+      </c>
+      <c r="E10" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6">
+        <v>44377</v>
+      </c>
+      <c r="B11" t="s">
+        <v>756</v>
+      </c>
+      <c r="C11" t="s">
+        <v>757</v>
+      </c>
+      <c r="D11" t="s">
+        <v>758</v>
+      </c>
+      <c r="E11" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6">
+        <v>46204</v>
+      </c>
+      <c r="B12" t="s">
+        <v>760</v>
+      </c>
+      <c r="C12" t="s">
+        <v>761</v>
+      </c>
+      <c r="D12" t="s">
+        <v>762</v>
+      </c>
+      <c r="E12" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6">
         <v>46174</v>
       </c>
-      <c r="B3" t="s">
-        <v>250</v>
-      </c>
-      <c r="C3" t="s">
-        <v>251</v>
-      </c>
-      <c r="D3" t="s">
-        <v>252</v>
-      </c>
-      <c r="E3" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
+      <c r="B13" t="s">
+        <v>764</v>
+      </c>
+      <c r="C13" t="s">
+        <v>765</v>
+      </c>
+      <c r="D13" t="s">
+        <v>766</v>
+      </c>
+      <c r="E13" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6">
+        <v>45658</v>
+      </c>
+      <c r="B14" t="s">
+        <v>768</v>
+      </c>
+      <c r="C14" t="s">
+        <v>769</v>
+      </c>
+      <c r="D14" t="s">
+        <v>770</v>
+      </c>
+      <c r="E14" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B15" t="s">
+        <v>772</v>
+      </c>
+      <c r="C15" t="s">
+        <v>773</v>
+      </c>
+      <c r="D15" t="s">
+        <v>774</v>
+      </c>
+      <c r="E15" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B16" t="s">
+        <v>776</v>
+      </c>
+      <c r="C16" t="s">
+        <v>777</v>
+      </c>
+      <c r="D16" t="s">
+        <v>778</v>
+      </c>
+      <c r="E16" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6">
+        <v>46082</v>
+      </c>
+      <c r="B17" t="s">
+        <v>780</v>
+      </c>
+      <c r="C17" t="s">
+        <v>781</v>
+      </c>
+      <c r="D17" t="s">
+        <v>782</v>
+      </c>
+      <c r="E17" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6">
         <v>44377</v>
       </c>
-      <c r="B4" t="s">
-        <v>254</v>
-      </c>
-      <c r="C4" t="s">
-        <v>255</v>
-      </c>
-      <c r="D4" t="s">
-        <v>256</v>
-      </c>
-      <c r="E4" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2">
+      <c r="B18" t="s">
+        <v>784</v>
+      </c>
+      <c r="C18" t="s">
+        <v>785</v>
+      </c>
+      <c r="D18" t="s">
+        <v>786</v>
+      </c>
+      <c r="E18" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6">
+        <v>45473</v>
+      </c>
+      <c r="B19" t="s">
+        <v>788</v>
+      </c>
+      <c r="C19" t="s">
+        <v>789</v>
+      </c>
+      <c r="D19" t="s">
+        <v>790</v>
+      </c>
+      <c r="E19" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6">
+        <v>44561</v>
+      </c>
+      <c r="B20" t="s">
+        <v>792</v>
+      </c>
+      <c r="C20" t="s">
+        <v>793</v>
+      </c>
+      <c r="D20" t="s">
+        <v>794</v>
+      </c>
+      <c r="E20" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6">
+        <v>44377</v>
+      </c>
+      <c r="B21" t="s">
+        <v>796</v>
+      </c>
+      <c r="C21" t="s">
+        <v>797</v>
+      </c>
+      <c r="D21" t="s">
+        <v>798</v>
+      </c>
+      <c r="E21" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6">
+        <v>45473</v>
+      </c>
+      <c r="B22" t="s">
+        <v>800</v>
+      </c>
+      <c r="C22" t="s">
+        <v>801</v>
+      </c>
+      <c r="D22" t="s">
+        <v>802</v>
+      </c>
+      <c r="E22" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B23" t="s">
+        <v>804</v>
+      </c>
+      <c r="C23" t="s">
+        <v>805</v>
+      </c>
+      <c r="D23" t="s">
+        <v>806</v>
+      </c>
+      <c r="E23" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6">
+        <v>44377</v>
+      </c>
+      <c r="B24" t="s">
+        <v>808</v>
+      </c>
+      <c r="C24" t="s">
+        <v>809</v>
+      </c>
+      <c r="D24" t="s">
+        <v>810</v>
+      </c>
+      <c r="E24" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6">
+        <v>44377</v>
+      </c>
+      <c r="B25" t="s">
+        <v>812</v>
+      </c>
+      <c r="C25" t="s">
+        <v>813</v>
+      </c>
+      <c r="D25" t="s">
+        <v>814</v>
+      </c>
+      <c r="E25" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6">
+        <v>46082</v>
+      </c>
+      <c r="B26" t="s">
+        <v>816</v>
+      </c>
+      <c r="C26" t="s">
+        <v>817</v>
+      </c>
+      <c r="D26" t="s">
+        <v>818</v>
+      </c>
+      <c r="E26" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B27" t="s">
+        <v>820</v>
+      </c>
+      <c r="C27" t="s">
+        <v>821</v>
+      </c>
+      <c r="D27" t="s">
+        <v>822</v>
+      </c>
+      <c r="E27" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6">
+        <v>44561</v>
+      </c>
+      <c r="B28" t="s">
+        <v>824</v>
+      </c>
+      <c r="C28" t="s">
+        <v>825</v>
+      </c>
+      <c r="D28" t="s">
+        <v>826</v>
+      </c>
+      <c r="E28" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B29" t="s">
+        <v>828</v>
+      </c>
+      <c r="C29" t="s">
+        <v>829</v>
+      </c>
+      <c r="D29" t="s">
+        <v>830</v>
+      </c>
+      <c r="E29" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6">
+        <v>45473</v>
+      </c>
+      <c r="B30" t="s">
+        <v>832</v>
+      </c>
+      <c r="C30" t="s">
+        <v>833</v>
+      </c>
+      <c r="D30" t="s">
+        <v>834</v>
+      </c>
+      <c r="E30" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6">
+        <v>44377</v>
+      </c>
+      <c r="B31" t="s">
+        <v>836</v>
+      </c>
+      <c r="C31" t="s">
+        <v>837</v>
+      </c>
+      <c r="D31" t="s">
+        <v>838</v>
+      </c>
+      <c r="E31" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B32" t="s">
+        <v>840</v>
+      </c>
+      <c r="C32" t="s">
+        <v>841</v>
+      </c>
+      <c r="D32" t="s">
+        <v>842</v>
+      </c>
+      <c r="E32" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B33" t="s">
+        <v>844</v>
+      </c>
+      <c r="C33" t="s">
+        <v>845</v>
+      </c>
+      <c r="D33" t="s">
+        <v>846</v>
+      </c>
+      <c r="E33" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6">
+        <v>44377</v>
+      </c>
+      <c r="B34" t="s">
+        <v>848</v>
+      </c>
+      <c r="C34" t="s">
+        <v>849</v>
+      </c>
+      <c r="D34" t="s">
+        <v>850</v>
+      </c>
+      <c r="E34" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B35" t="s">
+        <v>852</v>
+      </c>
+      <c r="C35" t="s">
+        <v>853</v>
+      </c>
+      <c r="D35" t="s">
+        <v>854</v>
+      </c>
+      <c r="E35" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6">
+        <v>46022</v>
+      </c>
+      <c r="B36" t="s">
+        <v>856</v>
+      </c>
+      <c r="C36" t="s">
+        <v>857</v>
+      </c>
+      <c r="D36" t="s">
+        <v>858</v>
+      </c>
+      <c r="E36" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B37" t="s">
+        <v>860</v>
+      </c>
+      <c r="C37" t="s">
+        <v>861</v>
+      </c>
+      <c r="D37" t="s">
+        <v>862</v>
+      </c>
+      <c r="E37" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6">
+        <v>45473</v>
+      </c>
+      <c r="B38" t="s">
+        <v>864</v>
+      </c>
+      <c r="C38" t="s">
+        <v>865</v>
+      </c>
+      <c r="D38" t="s">
+        <v>866</v>
+      </c>
+      <c r="E38" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6">
+        <v>46022</v>
+      </c>
+      <c r="B39" t="s">
+        <v>868</v>
+      </c>
+      <c r="C39" t="s">
+        <v>869</v>
+      </c>
+      <c r="D39" t="s">
+        <v>870</v>
+      </c>
+      <c r="E39" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6">
+        <v>44377</v>
+      </c>
+      <c r="B40" t="s">
+        <v>872</v>
+      </c>
+      <c r="C40" t="s">
+        <v>873</v>
+      </c>
+      <c r="D40" t="s">
+        <v>874</v>
+      </c>
+      <c r="E40" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6">
+        <v>46204</v>
+      </c>
+      <c r="B41" t="s">
+        <v>876</v>
+      </c>
+      <c r="C41" t="s">
+        <v>877</v>
+      </c>
+      <c r="D41" t="s">
+        <v>878</v>
+      </c>
+      <c r="E41" t="s">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6">
+        <v>44377</v>
+      </c>
+      <c r="B42" t="s">
+        <v>880</v>
+      </c>
+      <c r="C42" t="s">
+        <v>881</v>
+      </c>
+      <c r="D42" t="s">
+        <v>882</v>
+      </c>
+      <c r="E42" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6">
+        <v>44377</v>
+      </c>
+      <c r="B43" t="s">
+        <v>884</v>
+      </c>
+      <c r="C43" t="s">
+        <v>885</v>
+      </c>
+      <c r="D43" t="s">
+        <v>886</v>
+      </c>
+      <c r="E43" t="s">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6">
+        <v>45473</v>
+      </c>
+      <c r="B44" t="s">
+        <v>888</v>
+      </c>
+      <c r="C44" t="s">
+        <v>889</v>
+      </c>
+      <c r="D44" t="s">
+        <v>890</v>
+      </c>
+      <c r="E44" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6">
         <v>45658</v>
       </c>
-      <c r="B5" t="s">
-        <v>258</v>
-      </c>
-      <c r="C5" t="s">
-        <v>259</v>
-      </c>
-      <c r="D5" t="s">
-        <v>260</v>
-      </c>
-      <c r="E5" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
+      <c r="B45" t="s">
+        <v>892</v>
+      </c>
+      <c r="C45" t="s">
+        <v>893</v>
+      </c>
+      <c r="D45" t="s">
+        <v>894</v>
+      </c>
+      <c r="E45" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B46" t="s">
+        <v>896</v>
+      </c>
+      <c r="C46" t="s">
+        <v>897</v>
+      </c>
+      <c r="D46" t="s">
+        <v>898</v>
+      </c>
+      <c r="E46" t="s">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B47" t="s">
+        <v>900</v>
+      </c>
+      <c r="C47" t="s">
+        <v>901</v>
+      </c>
+      <c r="D47" t="s">
+        <v>902</v>
+      </c>
+      <c r="E47" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6">
         <v>44377</v>
       </c>
-      <c r="B6" t="s">
-        <v>262</v>
-      </c>
-      <c r="C6" t="s">
-        <v>263</v>
-      </c>
-      <c r="D6" t="s">
-        <v>264</v>
-      </c>
-      <c r="E6" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
+      <c r="B48" t="s">
+        <v>904</v>
+      </c>
+      <c r="C48" t="s">
+        <v>905</v>
+      </c>
+      <c r="D48" t="s">
+        <v>906</v>
+      </c>
+      <c r="E48" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6">
+        <v>46082</v>
+      </c>
+      <c r="B49" t="s">
+        <v>908</v>
+      </c>
+      <c r="C49" t="s">
+        <v>909</v>
+      </c>
+      <c r="D49" t="s">
+        <v>910</v>
+      </c>
+      <c r="E49" t="s">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B50" t="s">
+        <v>912</v>
+      </c>
+      <c r="C50" t="s">
+        <v>913</v>
+      </c>
+      <c r="D50" t="s">
+        <v>914</v>
+      </c>
+      <c r="E50" t="s">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B51" t="s">
+        <v>916</v>
+      </c>
+      <c r="C51" t="s">
+        <v>917</v>
+      </c>
+      <c r="D51" t="s">
+        <v>918</v>
+      </c>
+      <c r="E51" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6">
+        <v>45838</v>
+      </c>
+      <c r="B52" t="s">
+        <v>920</v>
+      </c>
+      <c r="C52" t="s">
+        <v>921</v>
+      </c>
+      <c r="D52" t="s">
+        <v>922</v>
+      </c>
+      <c r="E52" t="s">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6">
+        <v>45658</v>
+      </c>
+      <c r="B53" t="s">
+        <v>924</v>
+      </c>
+      <c r="C53" t="s">
+        <v>925</v>
+      </c>
+      <c r="D53" t="s">
+        <v>926</v>
+      </c>
+      <c r="E53" t="s">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6">
+        <v>46022</v>
+      </c>
+      <c r="B54" t="s">
+        <v>928</v>
+      </c>
+      <c r="C54" t="s">
+        <v>929</v>
+      </c>
+      <c r="D54" t="s">
+        <v>930</v>
+      </c>
+      <c r="E54" t="s">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B55" t="s">
+        <v>932</v>
+      </c>
+      <c r="C55" t="s">
+        <v>933</v>
+      </c>
+      <c r="D55" t="s">
+        <v>934</v>
+      </c>
+      <c r="E55" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6">
+        <v>46022</v>
+      </c>
+      <c r="B56" t="s">
+        <v>936</v>
+      </c>
+      <c r="C56" t="s">
+        <v>937</v>
+      </c>
+      <c r="D56" t="s">
+        <v>938</v>
+      </c>
+      <c r="E56" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6">
+        <v>46204</v>
+      </c>
+      <c r="B57" t="s">
+        <v>940</v>
+      </c>
+      <c r="C57" t="s">
+        <v>941</v>
+      </c>
+      <c r="D57" t="s">
+        <v>942</v>
+      </c>
+      <c r="E57" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6">
         <v>45473</v>
       </c>
-      <c r="B7" t="s">
-        <v>266</v>
-      </c>
-      <c r="C7" t="s">
-        <v>267</v>
-      </c>
-      <c r="D7" t="s">
-        <v>268</v>
-      </c>
-      <c r="E7" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>46082</v>
-      </c>
-      <c r="B8" t="s">
-        <v>270</v>
-      </c>
-      <c r="C8" t="s">
-        <v>271</v>
-      </c>
-      <c r="D8" t="s">
-        <v>272</v>
-      </c>
-      <c r="E8" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>46143</v>
-      </c>
-      <c r="B9" t="s">
-        <v>274</v>
-      </c>
-      <c r="C9" t="s">
-        <v>275</v>
-      </c>
-      <c r="D9" t="s">
-        <v>276</v>
-      </c>
-      <c r="E9" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2">
-        <v>46022</v>
-      </c>
-      <c r="B10" t="s">
-        <v>278</v>
-      </c>
-      <c r="C10" t="s">
-        <v>279</v>
-      </c>
-      <c r="D10" t="s">
-        <v>280</v>
-      </c>
-      <c r="E10" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2">
-        <v>45473</v>
-      </c>
-      <c r="B11" t="s">
-        <v>282</v>
-      </c>
-      <c r="C11" t="s">
-        <v>283</v>
-      </c>
-      <c r="D11" t="s">
-        <v>284</v>
-      </c>
-      <c r="E11" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2">
-        <v>44377</v>
-      </c>
-      <c r="B12" t="s">
-        <v>286</v>
-      </c>
-      <c r="C12" t="s">
-        <v>287</v>
-      </c>
-      <c r="D12" t="s">
-        <v>288</v>
-      </c>
-      <c r="E12" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2">
-        <v>46082</v>
-      </c>
-      <c r="B13" t="s">
-        <v>290</v>
-      </c>
-      <c r="C13" t="s">
-        <v>291</v>
-      </c>
-      <c r="D13" t="s">
-        <v>292</v>
-      </c>
-      <c r="E13" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2">
-        <v>45658</v>
-      </c>
-      <c r="B14" t="s">
-        <v>294</v>
-      </c>
-      <c r="C14" t="s">
-        <v>295</v>
-      </c>
-      <c r="D14" t="s">
-        <v>296</v>
-      </c>
-      <c r="E14" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2">
-        <v>46082</v>
-      </c>
-      <c r="B15" t="s">
-        <v>298</v>
-      </c>
-      <c r="C15" t="s">
-        <v>299</v>
-      </c>
-      <c r="D15" t="s">
-        <v>300</v>
-      </c>
-      <c r="E15" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2">
-        <v>44377</v>
-      </c>
-      <c r="B16" t="s">
-        <v>302</v>
-      </c>
-      <c r="C16" t="s">
-        <v>303</v>
-      </c>
-      <c r="D16" t="s">
-        <v>304</v>
-      </c>
-      <c r="E16" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2">
-        <v>46082</v>
-      </c>
-      <c r="B17" t="s">
-        <v>306</v>
-      </c>
-      <c r="C17" t="s">
-        <v>307</v>
-      </c>
-      <c r="D17" t="s">
-        <v>308</v>
-      </c>
-      <c r="E17" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2">
-        <v>45473</v>
-      </c>
-      <c r="B18" t="s">
-        <v>310</v>
-      </c>
-      <c r="C18" t="s">
-        <v>311</v>
-      </c>
-      <c r="D18" t="s">
-        <v>312</v>
-      </c>
-      <c r="E18" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2">
-        <v>44561</v>
-      </c>
-      <c r="B19" t="s">
-        <v>314</v>
-      </c>
-      <c r="C19" t="s">
-        <v>315</v>
-      </c>
-      <c r="D19" t="s">
-        <v>316</v>
-      </c>
-      <c r="E19" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2">
-        <v>44377</v>
-      </c>
-      <c r="B20" t="s">
-        <v>318</v>
-      </c>
-      <c r="C20" t="s">
-        <v>319</v>
-      </c>
-      <c r="D20" t="s">
-        <v>320</v>
-      </c>
-      <c r="E20" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2">
-        <v>45473</v>
-      </c>
-      <c r="B21" t="s">
-        <v>322</v>
-      </c>
-      <c r="C21" t="s">
-        <v>323</v>
-      </c>
-      <c r="D21" t="s">
-        <v>324</v>
-      </c>
-      <c r="E21" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2">
+      <c r="B58" t="s">
+        <v>944</v>
+      </c>
+      <c r="C58" t="s">
+        <v>945</v>
+      </c>
+      <c r="D58" t="s">
+        <v>946</v>
+      </c>
+      <c r="E58" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6">
         <v>46174</v>
       </c>
-      <c r="B22" t="s">
-        <v>326</v>
-      </c>
-      <c r="C22" t="s">
-        <v>327</v>
-      </c>
-      <c r="D22" t="s">
-        <v>328</v>
-      </c>
-      <c r="E22" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2">
-        <v>46082</v>
-      </c>
-      <c r="B23" t="s">
-        <v>330</v>
-      </c>
-      <c r="C23" t="s">
-        <v>331</v>
-      </c>
-      <c r="D23" t="s">
-        <v>332</v>
-      </c>
-      <c r="E23" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2">
-        <v>44377</v>
-      </c>
-      <c r="B24" t="s">
-        <v>334</v>
-      </c>
-      <c r="C24" t="s">
-        <v>335</v>
-      </c>
-      <c r="D24" t="s">
-        <v>336</v>
-      </c>
-      <c r="E24" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2">
-        <v>44377</v>
-      </c>
-      <c r="B25" t="s">
-        <v>338</v>
-      </c>
-      <c r="C25" t="s">
-        <v>339</v>
-      </c>
-      <c r="D25" t="s">
-        <v>340</v>
-      </c>
-      <c r="E25" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2">
-        <v>46082</v>
-      </c>
-      <c r="B26" t="s">
-        <v>342</v>
-      </c>
-      <c r="C26" t="s">
-        <v>343</v>
-      </c>
-      <c r="D26" t="s">
-        <v>344</v>
-      </c>
-      <c r="E26" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2">
-        <v>46174</v>
-      </c>
-      <c r="B27" t="s">
-        <v>346</v>
-      </c>
-      <c r="C27" t="s">
-        <v>347</v>
-      </c>
-      <c r="D27" t="s">
-        <v>348</v>
-      </c>
-      <c r="E27" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2">
-        <v>46174</v>
-      </c>
-      <c r="B28" t="s">
-        <v>350</v>
-      </c>
-      <c r="C28" t="s">
-        <v>351</v>
-      </c>
-      <c r="D28" t="s">
-        <v>352</v>
-      </c>
-      <c r="E28" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2">
-        <v>44561</v>
-      </c>
-      <c r="B29" t="s">
-        <v>354</v>
-      </c>
-      <c r="C29" t="s">
-        <v>355</v>
-      </c>
-      <c r="D29" t="s">
-        <v>356</v>
-      </c>
-      <c r="E29" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2">
-        <v>46174</v>
-      </c>
-      <c r="B30" t="s">
-        <v>358</v>
-      </c>
-      <c r="C30" t="s">
-        <v>359</v>
-      </c>
-      <c r="D30" t="s">
-        <v>360</v>
-      </c>
-      <c r="E30" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2">
-        <v>45473</v>
-      </c>
-      <c r="B31" t="s">
-        <v>362</v>
-      </c>
-      <c r="C31" t="s">
-        <v>363</v>
-      </c>
-      <c r="D31" t="s">
-        <v>364</v>
-      </c>
-      <c r="E31" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2">
-        <v>44377</v>
-      </c>
-      <c r="B32" t="s">
-        <v>366</v>
-      </c>
-      <c r="C32" t="s">
-        <v>367</v>
-      </c>
-      <c r="D32" t="s">
-        <v>368</v>
-      </c>
-      <c r="E32" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2">
-        <v>46174</v>
-      </c>
-      <c r="B33" t="s">
-        <v>370</v>
-      </c>
-      <c r="C33" t="s">
-        <v>371</v>
-      </c>
-      <c r="D33" t="s">
-        <v>372</v>
-      </c>
-      <c r="E33" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2">
-        <v>44377</v>
-      </c>
-      <c r="B34" t="s">
-        <v>374</v>
-      </c>
-      <c r="C34" t="s">
-        <v>375</v>
-      </c>
-      <c r="D34" t="s">
-        <v>376</v>
-      </c>
-      <c r="E34" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2">
-        <v>46082</v>
-      </c>
-      <c r="B35" t="s">
-        <v>378</v>
-      </c>
-      <c r="C35" t="s">
-        <v>379</v>
-      </c>
-      <c r="D35" t="s">
-        <v>380</v>
-      </c>
-      <c r="E35" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2">
-        <v>46022</v>
-      </c>
-      <c r="B36" t="s">
-        <v>382</v>
-      </c>
-      <c r="C36" t="s">
-        <v>383</v>
-      </c>
-      <c r="D36" t="s">
-        <v>384</v>
-      </c>
-      <c r="E36" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2">
-        <v>46082</v>
-      </c>
-      <c r="B37" t="s">
-        <v>386</v>
-      </c>
-      <c r="C37" t="s">
-        <v>387</v>
-      </c>
-      <c r="D37" t="s">
-        <v>388</v>
-      </c>
-      <c r="E37" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2">
-        <v>45473</v>
-      </c>
-      <c r="B38" t="s">
-        <v>390</v>
-      </c>
-      <c r="C38" t="s">
-        <v>391</v>
-      </c>
-      <c r="D38" t="s">
-        <v>392</v>
-      </c>
-      <c r="E38" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2">
-        <v>46022</v>
-      </c>
-      <c r="B39" t="s">
-        <v>394</v>
-      </c>
-      <c r="C39" t="s">
-        <v>395</v>
-      </c>
-      <c r="D39" t="s">
-        <v>396</v>
-      </c>
-      <c r="E39" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2">
-        <v>44377</v>
-      </c>
-      <c r="B40" t="s">
-        <v>398</v>
-      </c>
-      <c r="C40" t="s">
-        <v>399</v>
-      </c>
-      <c r="D40" t="s">
-        <v>400</v>
-      </c>
-      <c r="E40" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2">
-        <v>44377</v>
-      </c>
-      <c r="B41" t="s">
-        <v>402</v>
-      </c>
-      <c r="C41" t="s">
-        <v>403</v>
-      </c>
-      <c r="D41" t="s">
-        <v>404</v>
-      </c>
-      <c r="E41" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2">
-        <v>44377</v>
-      </c>
-      <c r="B42" t="s">
-        <v>406</v>
-      </c>
-      <c r="C42" t="s">
-        <v>407</v>
-      </c>
-      <c r="D42" t="s">
-        <v>408</v>
-      </c>
-      <c r="E42" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2">
-        <v>45473</v>
-      </c>
-      <c r="B43" t="s">
-        <v>410</v>
-      </c>
-      <c r="C43" t="s">
-        <v>411</v>
-      </c>
-      <c r="D43" t="s">
-        <v>412</v>
-      </c>
-      <c r="E43" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2">
-        <v>46174</v>
-      </c>
-      <c r="B44" t="s">
-        <v>414</v>
-      </c>
-      <c r="C44" t="s">
-        <v>415</v>
-      </c>
-      <c r="D44" t="s">
-        <v>416</v>
-      </c>
-      <c r="E44" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2">
-        <v>45658</v>
-      </c>
-      <c r="B45" t="s">
-        <v>418</v>
-      </c>
-      <c r="C45" t="s">
-        <v>419</v>
-      </c>
-      <c r="D45" t="s">
-        <v>420</v>
-      </c>
-      <c r="E45" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2">
-        <v>46174</v>
-      </c>
-      <c r="B46" t="s">
-        <v>422</v>
-      </c>
-      <c r="C46" t="s">
-        <v>423</v>
-      </c>
-      <c r="D46" t="s">
-        <v>424</v>
-      </c>
-      <c r="E46" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2">
-        <v>46082</v>
-      </c>
-      <c r="B47" t="s">
-        <v>426</v>
-      </c>
-      <c r="C47" t="s">
-        <v>427</v>
-      </c>
-      <c r="D47" t="s">
-        <v>428</v>
-      </c>
-      <c r="E47" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2">
-        <v>44377</v>
-      </c>
-      <c r="B48" t="s">
-        <v>430</v>
-      </c>
-      <c r="C48" t="s">
-        <v>431</v>
-      </c>
-      <c r="D48" t="s">
-        <v>432</v>
-      </c>
-      <c r="E48" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2">
-        <v>46082</v>
-      </c>
-      <c r="B49" t="s">
-        <v>434</v>
-      </c>
-      <c r="C49" t="s">
-        <v>435</v>
-      </c>
-      <c r="D49" t="s">
-        <v>436</v>
-      </c>
-      <c r="E49" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2">
-        <v>46174</v>
-      </c>
-      <c r="B50" t="s">
-        <v>438</v>
-      </c>
-      <c r="C50" t="s">
-        <v>439</v>
-      </c>
-      <c r="D50" t="s">
-        <v>440</v>
-      </c>
-      <c r="E50" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2">
-        <v>46174</v>
-      </c>
-      <c r="B51" t="s">
-        <v>442</v>
-      </c>
-      <c r="C51" t="s">
-        <v>443</v>
-      </c>
-      <c r="D51" t="s">
-        <v>444</v>
-      </c>
-      <c r="E51" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2">
-        <v>45838</v>
-      </c>
-      <c r="B52" t="s">
-        <v>446</v>
-      </c>
-      <c r="C52" t="s">
-        <v>447</v>
-      </c>
-      <c r="D52" t="s">
-        <v>448</v>
-      </c>
-      <c r="E52" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2">
-        <v>45658</v>
-      </c>
-      <c r="B53" t="s">
-        <v>450</v>
-      </c>
-      <c r="C53" t="s">
-        <v>451</v>
-      </c>
-      <c r="D53" t="s">
-        <v>452</v>
-      </c>
-      <c r="E53" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2">
-        <v>46022</v>
-      </c>
-      <c r="B54" t="s">
-        <v>454</v>
-      </c>
-      <c r="C54" t="s">
-        <v>455</v>
-      </c>
-      <c r="D54" t="s">
-        <v>456</v>
-      </c>
-      <c r="E54" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2">
-        <v>46022</v>
-      </c>
-      <c r="B55" t="s">
-        <v>458</v>
-      </c>
-      <c r="C55" t="s">
-        <v>459</v>
-      </c>
-      <c r="D55" t="s">
-        <v>460</v>
-      </c>
-      <c r="E55" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2">
-        <v>46143</v>
-      </c>
-      <c r="B56" t="s">
-        <v>462</v>
-      </c>
-      <c r="C56" t="s">
-        <v>463</v>
-      </c>
-      <c r="D56" t="s">
-        <v>464</v>
-      </c>
-      <c r="E56" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2">
-        <v>45473</v>
-      </c>
-      <c r="B57" t="s">
-        <v>466</v>
-      </c>
-      <c r="C57" t="s">
-        <v>467</v>
-      </c>
-      <c r="D57" t="s">
-        <v>468</v>
-      </c>
-      <c r="E57" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2">
-        <v>46082</v>
-      </c>
-      <c r="B58" t="s">
-        <v>470</v>
-      </c>
-      <c r="C58" t="s">
-        <v>471</v>
-      </c>
-      <c r="D58" t="s">
-        <v>472</v>
-      </c>
-      <c r="E58" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2">
-        <v>46174</v>
-      </c>
       <c r="B59" t="s">
-        <v>474</v>
+        <v>948</v>
       </c>
       <c r="C59" t="s">
-        <v>475</v>
+        <v>949</v>
       </c>
       <c r="D59" t="s">
-        <v>476</v>
+        <v>950</v>
       </c>
       <c r="E59" t="s">
-        <v>477</v>
+        <v>951</v>
       </c>
     </row>
   </sheetData>

</xml_diff>